<commit_message>
update GMT calcs sheet
</commit_message>
<xml_diff>
--- a/Document/report/ofl_report/GMT_calcs.xlsx
+++ b/Document/report/ofl_report/GMT_calcs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jason.Cope\Documents\Github\REBS-2025\Document\report\ofl_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B845A900-25E2-4D8B-A958-22C01FEC3EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8024D22-43E3-4407-B7D9-7D49E2D32960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{221927F3-A3BC-49E5-8350-92FAF4A860D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{221927F3-A3BC-49E5-8350-92FAF4A860D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Catch calcs" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="7">
   <si>
     <t>Year</t>
   </si>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t>519 mt for 2027-2028</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
 </sst>
 </file>
@@ -1344,8 +1341,8 @@
       <c r="A4" s="1">
         <v>2025</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
+      <c r="B4" s="3">
+        <v>954.66099999999994</v>
       </c>
       <c r="C4" s="1">
         <v>155.1</v>
@@ -1361,8 +1358,8 @@
       <c r="A5" s="1">
         <v>2026</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>7</v>
+      <c r="B5" s="3">
+        <v>960.51400000000001</v>
       </c>
       <c r="C5" s="1">
         <v>186.7</v>
@@ -1378,8 +1375,8 @@
       <c r="A6" s="1">
         <v>2027</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>7</v>
+      <c r="B6" s="3">
+        <v>965.50599999999997</v>
       </c>
       <c r="C6" s="1">
         <v>300</v>
@@ -1395,8 +1392,8 @@
       <c r="A7" s="1">
         <v>2028</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>7</v>
+      <c r="B7" s="3">
+        <v>967.44100000000003</v>
       </c>
       <c r="C7" s="1">
         <v>300</v>
@@ -1570,8 +1567,8 @@
       <c r="A19" s="1">
         <v>2025</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>7</v>
+      <c r="B19" s="3">
+        <v>954.66099999999994</v>
       </c>
       <c r="C19" s="1">
         <v>155.1</v>
@@ -1587,8 +1584,8 @@
       <c r="A20" s="1">
         <v>2026</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>7</v>
+      <c r="B20" s="3">
+        <v>960.51400000000001</v>
       </c>
       <c r="C20" s="1">
         <v>186.7</v>
@@ -1604,8 +1601,8 @@
       <c r="A21" s="1">
         <v>2027</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>7</v>
+      <c r="B21" s="3">
+        <v>965.50599999999997</v>
       </c>
       <c r="C21" s="1">
         <v>519</v>
@@ -1621,8 +1618,8 @@
       <c r="A22" s="1">
         <v>2028</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>7</v>
+      <c r="B22" s="3">
+        <v>962.18299999999999</v>
       </c>
       <c r="C22" s="1">
         <v>519</v>

</xml_diff>